<commit_message>
Weight optimization for different parts
</commit_message>
<xml_diff>
--- a/evaluations/classification/classification_results_global_embedding.xlsx
+++ b/evaluations/classification/classification_results_global_embedding.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U19"/>
+  <dimension ref="A1:W21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,6 +534,16 @@
           <t>F-1 Score</t>
         </is>
       </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Use Shape</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Dataset Type</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -605,6 +615,8 @@
       <c r="U2" t="n">
         <v>0.8248</v>
       </c>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -676,6 +688,8 @@
       <c r="U3" t="n">
         <v>0.883</v>
       </c>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -747,6 +761,8 @@
       <c r="U4" t="n">
         <v>0.052</v>
       </c>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -818,6 +834,8 @@
       <c r="U5" t="n">
         <v>0.08699999999999999</v>
       </c>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -889,6 +907,8 @@
       <c r="U6" t="n">
         <v>0.9474</v>
       </c>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -960,6 +980,8 @@
       <c r="U7" t="n">
         <v>0.9847</v>
       </c>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1031,6 +1053,8 @@
       <c r="U8" t="n">
         <v>0.5244</v>
       </c>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1102,6 +1126,8 @@
       <c r="U9" t="n">
         <v>0.484</v>
       </c>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1173,6 +1199,8 @@
       <c r="U10" t="n">
         <v>0.6079</v>
       </c>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1244,6 +1272,8 @@
       <c r="U11" t="n">
         <v>0.5302</v>
       </c>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1315,6 +1345,8 @@
       <c r="U12" t="n">
         <v>0.6287</v>
       </c>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1386,6 +1418,8 @@
       <c r="U13" t="n">
         <v>0.8038</v>
       </c>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1457,6 +1491,8 @@
       <c r="U14" t="n">
         <v>0.1345</v>
       </c>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1528,18 +1564,20 @@
       <c r="U15" t="n">
         <v>0.1318</v>
       </c>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SealID</t>
+          <t>NyalaData</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1668</v>
+        <v>1498</v>
       </c>
       <c r="C16" t="n">
-        <v>55</v>
+        <v>227</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1547,13 +1585,13 @@
         </is>
       </c>
       <c r="E16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" t="b">
         <v>0</v>
       </c>
       <c r="G16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
         <v>256</v>
@@ -1588,29 +1626,37 @@
         <v>0</v>
       </c>
       <c r="R16" t="n">
-        <v>5.68</v>
+        <v>6.91</v>
       </c>
       <c r="S16" t="n">
-        <v>0.6545</v>
+        <v>0.1503</v>
       </c>
       <c r="T16" t="n">
-        <v>0.7276</v>
+        <v>0.3671</v>
       </c>
       <c r="U16" t="n">
-        <v>0.6428</v>
+        <v>0.1288</v>
+      </c>
+      <c r="V16" t="n">
+        <v>1</v>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>WildlifeReID10k</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SealID</t>
+          <t>NyalaData</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1668</v>
+        <v>1498</v>
       </c>
       <c r="C17" t="n">
-        <v>55</v>
+        <v>227</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1618,7 +1664,7 @@
         </is>
       </c>
       <c r="E17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" t="b">
         <v>0</v>
@@ -1659,29 +1705,37 @@
         <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>5.44</v>
+        <v>9.98</v>
       </c>
       <c r="S17" t="n">
-        <v>0.7907</v>
+        <v>0.1503</v>
       </c>
       <c r="T17" t="n">
-        <v>0.8738</v>
+        <v>0.3671</v>
       </c>
       <c r="U17" t="n">
-        <v>0.7712</v>
+        <v>0.1288</v>
+      </c>
+      <c r="V17" t="n">
+        <v>1</v>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>WildlifeReID10k</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>StripeSpotter</t>
+          <t>SealID</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>655</v>
+        <v>1668</v>
       </c>
       <c r="C18" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1695,7 +1749,7 @@
         <v>0</v>
       </c>
       <c r="G18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H18" t="n">
         <v>256</v>
@@ -1730,29 +1784,31 @@
         <v>0</v>
       </c>
       <c r="R18" t="n">
-        <v>1.73</v>
+        <v>5.68</v>
       </c>
       <c r="S18" t="n">
-        <v>0.9826</v>
+        <v>0.6545</v>
       </c>
       <c r="T18" t="n">
-        <v>1</v>
+        <v>0.7276</v>
       </c>
       <c r="U18" t="n">
-        <v>0.9797</v>
-      </c>
+        <v>0.6428</v>
+      </c>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>StripeSpotter</t>
+          <t>SealID</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>655</v>
+        <v>1668</v>
       </c>
       <c r="C19" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1766,7 +1822,7 @@
         <v>0</v>
       </c>
       <c r="G19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
         <v>256</v>
@@ -1801,17 +1857,165 @@
         <v>0</v>
       </c>
       <c r="R19" t="n">
+        <v>5.44</v>
+      </c>
+      <c r="S19" t="n">
+        <v>0.7907</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0.8738</v>
+      </c>
+      <c r="U19" t="n">
+        <v>0.7712</v>
+      </c>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>StripeSpotter</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>655</v>
+      </c>
+      <c r="C20" t="n">
+        <v>43</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ensamble</t>
+        </is>
+      </c>
+      <c r="E20" t="b">
+        <v>0</v>
+      </c>
+      <c r="F20" t="b">
+        <v>0</v>
+      </c>
+      <c r="G20" t="b">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>256</v>
+      </c>
+      <c r="I20" t="n">
+        <v>128</v>
+      </c>
+      <c r="J20" t="b">
+        <v>1</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>RANSAC</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="M20" t="n">
+        <v>50</v>
+      </c>
+      <c r="N20" t="n">
+        <v>10</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P20" t="n">
+        <v>5000</v>
+      </c>
+      <c r="Q20" t="b">
+        <v>0</v>
+      </c>
+      <c r="R20" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="S20" t="n">
+        <v>0.9826</v>
+      </c>
+      <c r="T20" t="n">
+        <v>1</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0.9797</v>
+      </c>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>StripeSpotter</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>655</v>
+      </c>
+      <c r="C21" t="n">
+        <v>43</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>ensamble</t>
+        </is>
+      </c>
+      <c r="E21" t="b">
+        <v>0</v>
+      </c>
+      <c r="F21" t="b">
+        <v>0</v>
+      </c>
+      <c r="G21" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" t="n">
+        <v>256</v>
+      </c>
+      <c r="I21" t="n">
+        <v>128</v>
+      </c>
+      <c r="J21" t="b">
+        <v>1</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>RANSAC</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="M21" t="n">
+        <v>50</v>
+      </c>
+      <c r="N21" t="n">
+        <v>10</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P21" t="n">
+        <v>5000</v>
+      </c>
+      <c r="Q21" t="b">
+        <v>0</v>
+      </c>
+      <c r="R21" t="n">
         <v>1.54</v>
       </c>
-      <c r="S19" t="n">
+      <c r="S21" t="n">
         <v>0.9391</v>
       </c>
-      <c r="T19" t="n">
+      <c r="T21" t="n">
         <v>0.9478</v>
       </c>
-      <c r="U19" t="n">
+      <c r="U21" t="n">
         <v>0.9331</v>
       </c>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>